<commit_message>
fix(reports): fold the arrow to a word and keep the em dash in PDFs; shorter auto-built line names
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/acceptance/EXP-2026-0001_Elaine-Xin-Yu-Khoo.xlsx
+++ b/docs/acceptance/EXP-2026-0001_Elaine-Xin-Yu-Khoo.xlsx
@@ -88,7 +88,7 @@
     <t>Approved at</t>
   </si>
   <si>
-    <t>2026-09-18T07:06:23.994Z</t>
+    <t>2026-09-18T07:11:04.947Z</t>
   </si>
   <si>
     <t>Advances</t>
@@ -145,7 +145,7 @@
     <t>JW Marriott Mumbai Sahar</t>
   </si>
   <si>
-    <t>Accomodation Charges, CGST 9%- Rooms-(New), SGST 9%- Rooms-(New)</t>
+    <t>Accomodation Charges +2 more</t>
   </si>
   <si>
     <t>Client meetings, Mumbai office</t>
@@ -166,7 +166,7 @@
     <t>R1</t>
   </si>
   <si>
-    <t>Upsell Breakfast-996331, JW Cafe CGST 9%, JW Cafe SGST 9%</t>
+    <t>Upsell Breakfast-996331 +2 more</t>
   </si>
   <si>
     <t>Meals</t>
@@ -175,7 +175,7 @@
     <t>Courtyard By Marriott Pune Chakan</t>
   </si>
   <si>
-    <t>Package, CGST ROOM 9%, SGST ROOM 9%</t>
+    <t>Package +9 more</t>
   </si>
   <si>
     <t>Client site visit, Chakan plant</t>
@@ -184,19 +184,19 @@
     <t>R2</t>
   </si>
   <si>
-    <t>Standard Retail [NA Room] TAN SUAN KUAN #126=&gt;Khoo Elaine Xin Yu #110, CGST ROOM 9% [Add; udf.] TAN SUAN KUAN #126=&gt;Khoo Elaine Xin Yu #110, SGST ROOM 9% [Add; udf.] TAN SUAN KUAN #126=&gt;Khoo Elaine Xi</t>
-  </si>
-  <si>
-    <t>MoMo Cafe Dinner Food Room# 110 : CHECK# 11603486 [pbhun211], MoMo Cafe Dinner Soda Room# 110 : CHECK# 11603486 [pbhun211], CGST Momo Cafe F&amp;B 9% Room# 110 : CHECK# 11603486 [pbhun211]</t>
-  </si>
-  <si>
-    <t>MoMo Cafe Dinner Food Room# 128 : CHECK# 11603551 [pbhun211] TAN SUAN KUAN #126=&gt;Khoo Elaine Xin Yu #110, CGST Momo Cafe F&amp;B 9% Room# 126 : CHECK# 11603551 [pbhun211] TAN SUAN KUAN #126=&gt;Khoo Elaine X</t>
-  </si>
-  <si>
-    <t>INR→SGD 0.01341, European Central Bank reference rate for 1 Sep 2026, via Frankfurter, fetched 18 Sep 2026 15:06 SGT.</t>
-  </si>
-  <si>
-    <t>INR→SGD 0.01341, European Central Bank reference rate for 4 Sep 2026, via Frankfurter, fetched 18 Sep 2026 15:06 SGT.</t>
+    <t>Standard Retail [NA Room] TAN SUAN KUAN #126=&gt;Khoo Elaine Xin Yu #110 +7 more</t>
+  </si>
+  <si>
+    <t>MoMo Cafe Dinner Food Room# 110 : CHECK# 11603486 [pbhun211] +14 more</t>
+  </si>
+  <si>
+    <t>MoMo Cafe Dinner Food Room# 128 : CHECK# 11603551 [pbhun211] TAN SUAN KUAN #126= +5 more</t>
+  </si>
+  <si>
+    <t>INR→SGD 0.01341, European Central Bank reference rate for 1 Sep 2026, via Frankfurter, fetched 18 Sep 2026 15:11 SGT.</t>
+  </si>
+  <si>
+    <t>INR→SGD 0.01341, European Central Bank reference rate for 4 Sep 2026, via Frankfurter, fetched 18 Sep 2026 15:11 SGT.</t>
   </si>
   <si>
     <t>Policy: rate on the receipt date. Each line is converted and rounded to the cent; the total is the sum of the lines.</t>

</xml_diff>